<commit_message>
chore: sync excel data and deploy (2026-06-12 15:57)
</commit_message>
<xml_diff>
--- a/data/공모_260611.xlsx
+++ b/data/공모_260611.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
-          <t>725</t>
+          <t>698</t>
         </is>
       </c>
       <c r="Q5" s="10" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="S5" s="10" t="inlineStr">
         <is>
-          <t>-23</t>
+          <t>-13</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>7,332</t>
+          <t>6,743</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>1,428</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>5,513</t>
+          <t>5,401</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>86,594</t>
+          <t>84,466</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>226</t>
         </is>
       </c>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>-15,839</t>
+          <t>-16,106</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>3,156</t>
+          <t>900</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>5,136</t>
+          <t>5,112</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>25</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N7" s="10" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>30,458</t>
+          <t>26,998</t>
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="R7" s="10" t="inlineStr">
         <is>
-          <t>-72</t>
+          <t>-69</t>
         </is>
       </c>
       <c r="S7" s="10" t="inlineStr">
         <is>
-          <t>-2,549</t>
+          <t>-1,621</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>952</t>
+          <t>78</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>55</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
-          <t>31,742</t>
+          <t>30,785</t>
         </is>
       </c>
       <c r="Q8" s="10" t="inlineStr">
@@ -897,12 +897,12 @@
       </c>
       <c r="R8" s="10" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>519</t>
         </is>
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>11,492</t>
+          <t>11,633</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>1,166</t>
+          <t>1,027</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>1,166</t>
+          <t>1,027</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>518</t>
+          <t>408</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="P10" s="10" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>105</t>
         </is>
       </c>
       <c r="Q10" s="10" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="S10" s="10" t="inlineStr">
         <is>
-          <t>-64</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1108,12 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>4,132</t>
+          <t>3,246</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>194</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>2,366</t>
+          <t>658</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>47,110</t>
+          <t>44,478</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>4,664</t>
+          <t>4,523</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>8,587</t>
+          <t>7,398</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>5,026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N13" s="10" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>36,268</t>
+          <t>29,830</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="R13" s="10" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>409</t>
         </is>
       </c>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>12,090</t>
+          <t>8,357</t>
         </is>
       </c>
     </row>
@@ -1491,27 +1491,27 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>머스트자산운용</t>
+          <t>미래에셋자산운용</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>558,325</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9,905</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12,534</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>110,748</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -1521,22 +1521,22 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>1,664</t>
+          <t>4,732</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>78,333</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>158,568</t>
         </is>
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>610</t>
         </is>
       </c>
       <c r="K15" s="10" t="inlineStr">
@@ -1546,12 +1546,12 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,016</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15,316</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>1,664</t>
+          <t>962,087</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
@@ -1576,39 +1576,39 @@
       </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
-          <t>-8</t>
+          <t>1,445</t>
         </is>
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>-422</t>
+          <t>380,822</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>미래에셋자산운용</t>
+          <t>밸류시스템자산운용</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>1,135,474</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>23,778</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>33,206</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>124,714</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -1618,22 +1618,22 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>32,948</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>80,000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>261,378</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
-          <t>7,509</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K16" s="10" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="L16" s="10" t="inlineStr">
         <is>
-          <t>16,333</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M16" s="10" t="inlineStr">
         <is>
-          <t>75,085</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="P16" s="10" t="inlineStr">
         <is>
-          <t>1,790,425</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q16" s="10" t="inlineStr">
@@ -1673,39 +1673,39 @@
       </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
-          <t>-7,914</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S16" s="10" t="inlineStr">
         <is>
-          <t>557,333</t>
+          <t>-104</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>밸류시스템자산운용</t>
+          <t>베어링자산운용</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,799</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>78</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>626</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>127</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,648</t>
         </is>
       </c>
       <c r="Q17" s="10" t="inlineStr">
@@ -1770,39 +1770,39 @@
       </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6</t>
         </is>
       </c>
       <c r="S17" s="10" t="inlineStr">
         <is>
-          <t>-104</t>
+          <t>-258</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>베어링자산운용</t>
+          <t>브레인자산운용</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>5,799</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>461</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>626</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="P18" s="10" t="inlineStr">
         <is>
-          <t>7,584</t>
+          <t>461</t>
         </is>
       </c>
       <c r="Q18" s="10" t="inlineStr">
@@ -1867,39 +1867,39 @@
       </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="S18" s="10" t="inlineStr">
         <is>
-          <t>-826</t>
+          <t>108</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>브레인자산운용</t>
+          <t>브이아이자산운용</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,738</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,135</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,346</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32,005</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>206</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>38,466</t>
         </is>
       </c>
       <c r="Q19" s="10" t="inlineStr">
@@ -1964,39 +1964,39 @@
       </c>
       <c r="R19" s="10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1,159</t>
         </is>
       </c>
       <c r="S19" s="10" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>14,873</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>브이아이자산운용</t>
+          <t>브이아이피자산운용</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>2,022</t>
+          <t>4,918</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>602</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>2,135</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>2,388</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -2006,22 +2006,22 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>277</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>32,005</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J20" s="10" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="P20" s="10" t="inlineStr">
         <is>
-          <t>39,711</t>
+          <t>4,918</t>
         </is>
       </c>
       <c r="Q20" s="10" t="inlineStr">
@@ -2061,39 +2061,39 @@
       </c>
       <c r="R20" s="10" t="inlineStr">
         <is>
-          <t>1,153</t>
+          <t>-17</t>
         </is>
       </c>
       <c r="S20" s="10" t="inlineStr">
         <is>
-          <t>14,689</t>
+          <t>-1,096</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>브이아이피자산운용</t>
+          <t>브이자산운용</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>4,918</t>
+          <t>214</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>121</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>27</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
@@ -2103,17 +2103,17 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,302</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>81</t>
         </is>
       </c>
       <c r="J21" s="10" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="P21" s="10" t="inlineStr">
         <is>
-          <t>4,918</t>
+          <t>2,757</t>
         </is>
       </c>
       <c r="Q21" s="10" t="inlineStr">
@@ -2158,39 +2158,39 @@
       </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
-          <t>-17</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="S21" s="10" t="inlineStr">
         <is>
-          <t>-1,096</t>
+          <t>173</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>브이자산운용</t>
+          <t>비엔케이자산운용</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>1,471</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>427</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>1,820</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -2200,17 +2200,17 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>2,302</t>
+          <t>40,044</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>339</t>
+          <t>1,015</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="P22" s="10" t="inlineStr">
         <is>
-          <t>3,024</t>
+          <t>44,802</t>
         </is>
       </c>
       <c r="Q22" s="10" t="inlineStr">
@@ -2255,39 +2255,39 @@
       </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>-393</t>
         </is>
       </c>
       <c r="S22" s="10" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>12,961</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>비엔케이자산운용</t>
+          <t>삼성액티브자산운용</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>1,471</t>
+          <t>21,079</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>1,820</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
@@ -2297,17 +2297,17 @@
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>604</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>40,044</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t>1,015</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J23" s="10" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
-          <t>45,400</t>
+          <t>21,079</t>
         </is>
       </c>
       <c r="Q23" s="10" t="inlineStr">
@@ -2352,39 +2352,39 @@
       </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
-          <t>-393</t>
+          <t>723</t>
         </is>
       </c>
       <c r="S23" s="10" t="inlineStr">
         <is>
-          <t>12,946</t>
+          <t>11,144</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>삼성액티브자산운용</t>
+          <t>삼성자산운용</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>34,120</t>
+          <t>779,964</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>62</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>1,374</t>
+          <t>35,200</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>222,364</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -2394,22 +2394,22 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>486</t>
+          <t>5,179</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>209,336</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>475,866</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,105</t>
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="P24" s="10" t="inlineStr">
         <is>
-          <t>35,980</t>
+          <t>1,733,076</t>
         </is>
       </c>
       <c r="Q24" s="10" t="inlineStr">
@@ -2449,39 +2449,39 @@
       </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>18,005</t>
         </is>
       </c>
       <c r="S24" s="10" t="inlineStr">
         <is>
-          <t>21,059</t>
+          <t>689,192</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>삼성자산운용</t>
+          <t>슈로더자산운용</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>1,068,726</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>39,032</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>235,404</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -2491,22 +2491,22 @@
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>67,716</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t>214,421</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I25" s="10" t="inlineStr">
         <is>
-          <t>600,859</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J25" s="10" t="inlineStr">
         <is>
-          <t>5,282</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K25" s="10" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="M25" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N25" s="10" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="P25" s="10" t="inlineStr">
         <is>
-          <t>2,231,506</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q25" s="10" t="inlineStr">
@@ -2546,24 +2546,24 @@
       </c>
       <c r="R25" s="10" t="inlineStr">
         <is>
-          <t>12,342</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S25" s="10" t="inlineStr">
         <is>
-          <t>812,005</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>슈로더자산운용</t>
+          <t>스팍스자산운용</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>350</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>152</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="P26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>502</t>
         </is>
       </c>
       <c r="Q26" s="10" t="inlineStr">
@@ -2643,39 +2643,39 @@
       </c>
       <c r="R26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-4</t>
         </is>
       </c>
       <c r="S26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>스팍스자산운용</t>
+          <t>신영자산운용</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>17,769</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,181</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>6,894</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>894</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -2685,12 +2685,12 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>117</t>
         </is>
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>51,954</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="M27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,237</t>
         </is>
       </c>
       <c r="N27" s="10" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>80,047</t>
         </is>
       </c>
       <c r="Q27" s="10" t="inlineStr">
@@ -2740,39 +2740,39 @@
       </c>
       <c r="R27" s="10" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-496</t>
         </is>
       </c>
       <c r="S27" s="10" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>23,538</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>신영자산운용</t>
+          <t>신한자산운용</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>17,821</t>
+          <t>133,513</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>1,498</t>
+          <t>686</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>6,894</t>
+          <t>8,093</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>894</t>
+          <t>59,748</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -2782,17 +2782,17 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>1,415</t>
+          <t>187</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>51,954</t>
+          <t>127,065</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17,659</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
@@ -2812,12 +2812,12 @@
       </c>
       <c r="M28" s="10" t="inlineStr">
         <is>
-          <t>1,237</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N28" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>360</t>
         </is>
       </c>
       <c r="O28" s="10" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="P28" s="10" t="inlineStr">
         <is>
-          <t>81,714</t>
+          <t>347,311</t>
         </is>
       </c>
       <c r="Q28" s="10" t="inlineStr">
@@ -2837,39 +2837,39 @@
       </c>
       <c r="R28" s="10" t="inlineStr">
         <is>
-          <t>-499</t>
+          <t>6,150</t>
         </is>
       </c>
       <c r="S28" s="10" t="inlineStr">
         <is>
-          <t>23,630</t>
+          <t>123,859</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>신한자산운용</t>
+          <t>아이비케이자산운용</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>175,818</t>
+          <t>4,370</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>692</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>14,790</t>
+          <t>2,229</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>68,027</t>
+          <t>4,981</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>24,475</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>129,455</t>
+          <t>112,144</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>34,552</t>
+          <t>117</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr">
@@ -2904,17 +2904,17 @@
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
-          <t>939</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M29" s="10" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N29" s="10" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O29" s="10" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="P29" s="10" t="inlineStr">
         <is>
-          <t>449,180</t>
+          <t>123,949</t>
         </is>
       </c>
       <c r="Q29" s="10" t="inlineStr">
@@ -2934,39 +2934,39 @@
       </c>
       <c r="R29" s="10" t="inlineStr">
         <is>
-          <t>5,286</t>
+          <t>465</t>
         </is>
       </c>
       <c r="S29" s="10" t="inlineStr">
         <is>
-          <t>132,546</t>
+          <t>18,264</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>아이비케이자산운용</t>
+          <t>아이엠에셋자산운용</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>5,528</t>
+          <t>1,545</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>2,951</t>
+          <t>976</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>4,981</t>
+          <t>1,058</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -2976,17 +2976,17 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>3,542</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>115,005</t>
+          <t>15,721</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>142</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="P30" s="10" t="inlineStr">
         <is>
-          <t>132,160</t>
+          <t>19,442</t>
         </is>
       </c>
       <c r="Q30" s="10" t="inlineStr">
@@ -3031,39 +3031,39 @@
       </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t>449</t>
+          <t>678</t>
         </is>
       </c>
       <c r="S30" s="10" t="inlineStr">
         <is>
-          <t>19,471</t>
+          <t>-7,154</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>아이엠에셋자산운용</t>
+          <t>알파자산운용</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>274</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>976</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>1,058</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -3073,17 +3073,17 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>5,432</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>15,721</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J31" s="10" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="P31" s="10" t="inlineStr">
         <is>
-          <t>24,874</t>
+          <t>274</t>
         </is>
       </c>
       <c r="Q31" s="10" t="inlineStr">
@@ -3128,34 +3128,34 @@
       </c>
       <c r="R31" s="10" t="inlineStr">
         <is>
-          <t>675</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S31" s="10" t="inlineStr">
         <is>
-          <t>-6,236</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>알파자산운용</t>
+          <t>에셋플러스자산운용</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>2,488</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>182</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>616</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="P32" s="10" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>3,287</t>
         </is>
       </c>
       <c r="Q32" s="10" t="inlineStr">
@@ -3225,24 +3225,24 @@
       </c>
       <c r="R32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89</t>
         </is>
       </c>
       <c r="S32" s="10" t="inlineStr">
         <is>
-          <t>-42</t>
+          <t>-183</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>얼라이언스번스틴자산운용</t>
+          <t>에이치디씨자산운용</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>386</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -3252,12 +3252,12 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>945</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
@@ -3267,12 +3267,12 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>13,683</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>101</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="P33" s="10" t="inlineStr">
         <is>
-          <t>13,683</t>
+          <t>1,436</t>
         </is>
       </c>
       <c r="Q33" s="10" t="inlineStr">
@@ -3322,34 +3322,34 @@
       </c>
       <c r="R33" s="10" t="inlineStr">
         <is>
-          <t>-33</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="S33" s="10" t="inlineStr">
         <is>
-          <t>-4,569</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>에셋플러스자산운용</t>
+          <t>에이케이파트너스자산운용</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>11,444</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>182</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>883</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="P34" s="10" t="inlineStr">
         <is>
-          <t>12,509</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q34" s="10" t="inlineStr">
@@ -3419,39 +3419,39 @@
       </c>
       <c r="R34" s="10" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S34" s="10" t="inlineStr">
         <is>
-          <t>-559</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>에이치디씨자산운용</t>
+          <t>엔에이치아문디자산운용</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>416</t>
+          <t>79,748</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>945</t>
+          <t>4,184</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10,627</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
@@ -3461,17 +3461,17 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>357</t>
         </is>
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>101,898</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>16,756</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="P35" s="10" t="inlineStr">
         <is>
-          <t>1,472</t>
+          <t>213,825</t>
         </is>
       </c>
       <c r="Q35" s="10" t="inlineStr">
@@ -3516,39 +3516,39 @@
       </c>
       <c r="R35" s="10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-53</t>
         </is>
       </c>
       <c r="S35" s="10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>70,166</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>에이케이파트너스자산운용</t>
+          <t>우리자산운용</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9,600</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>110</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,748</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36,882</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
@@ -3558,12 +3558,12 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71</t>
         </is>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>170,295</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>94</t>
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="P36" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>221,801</t>
         </is>
       </c>
       <c r="Q36" s="10" t="inlineStr">
@@ -3613,39 +3613,39 @@
       </c>
       <c r="R36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5,913</t>
         </is>
       </c>
       <c r="S36" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>62,542</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>엔에이치아문디자산운용</t>
+          <t>웰컴자산운용</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>86,211</t>
+          <t>785</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>161</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>4,184</t>
+          <t>1,916</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>11,262</t>
+          <t>465</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
@@ -3655,17 +3655,17 @@
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>12,050</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>103,635</t>
+          <t>5,092</t>
         </is>
       </c>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>17,031</t>
+          <t>1,303</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="P37" s="10" t="inlineStr">
         <is>
-          <t>234,629</t>
+          <t>9,723</t>
         </is>
       </c>
       <c r="Q37" s="10" t="inlineStr">
@@ -3710,39 +3710,39 @@
       </c>
       <c r="R37" s="10" t="inlineStr">
         <is>
-          <t>-140</t>
+          <t>-302</t>
         </is>
       </c>
       <c r="S37" s="10" t="inlineStr">
         <is>
-          <t>72,732</t>
+          <t>3,500</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>우리자산운용</t>
+          <t>유경피에스지자산운용</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>11,661</t>
+          <t>160</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>124</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>9,093</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>36,885</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
@@ -3752,12 +3752,12 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>6,184</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>172,553</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="J38" s="10" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>1,060</t>
         </is>
       </c>
       <c r="K38" s="10" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="P38" s="10" t="inlineStr">
         <is>
-          <t>236,625</t>
+          <t>1,365</t>
         </is>
       </c>
       <c r="Q38" s="10" t="inlineStr">
@@ -3807,39 +3807,39 @@
       </c>
       <c r="R38" s="10" t="inlineStr">
         <is>
-          <t>5,864</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S38" s="10" t="inlineStr">
         <is>
-          <t>66,278</t>
+          <t>-40</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>웰컴자산운용</t>
+          <t>유리자산운용</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>785</t>
+          <t>779</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>161</t>
+          <t>92</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>1,916</t>
+          <t>1,054</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>465</t>
+          <t>1,796</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
@@ -3849,17 +3849,17 @@
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>583</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
         <is>
-          <t>5,092</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I39" s="10" t="inlineStr">
         <is>
-          <t>1,303</t>
+          <t>198</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
-          <t>9,723</t>
+          <t>4,502</t>
         </is>
       </c>
       <c r="Q39" s="10" t="inlineStr">
@@ -3904,39 +3904,39 @@
       </c>
       <c r="R39" s="10" t="inlineStr">
         <is>
-          <t>-302</t>
+          <t>-25</t>
         </is>
       </c>
       <c r="S39" s="10" t="inlineStr">
         <is>
-          <t>3,500</t>
+          <t>1,449</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>유경피에스지자산운용</t>
+          <t>유진자산운용</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>108</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>119</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2,144</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,413</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
@@ -3946,12 +3946,12 @@
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>163</t>
         </is>
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,440</t>
         </is>
       </c>
       <c r="I40" s="10" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="J40" s="10" t="inlineStr">
         <is>
-          <t>1,093</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K40" s="10" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="M40" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>947</t>
         </is>
       </c>
       <c r="N40" s="10" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="P40" s="10" t="inlineStr">
         <is>
-          <t>1,577</t>
+          <t>31,334</t>
         </is>
       </c>
       <c r="Q40" s="10" t="inlineStr">
@@ -4001,39 +4001,39 @@
       </c>
       <c r="R40" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-681</t>
         </is>
       </c>
       <c r="S40" s="10" t="inlineStr">
         <is>
-          <t>-67</t>
+          <t>-10,788</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>유리자산운용</t>
+          <t>이지스자산운용</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>4,255</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>3,118</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>1,796</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H41" s="10" t="inlineStr">
@@ -4053,12 +4053,12 @@
       </c>
       <c r="I41" s="10" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,210</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="P41" s="10" t="inlineStr">
         <is>
-          <t>10,042</t>
+          <t>1,210</t>
         </is>
       </c>
       <c r="Q41" s="10" t="inlineStr">
@@ -4098,39 +4098,39 @@
       </c>
       <c r="R41" s="10" t="inlineStr">
         <is>
-          <t>-22</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S41" s="10" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>유진자산운용</t>
+          <t>카디안자산운용</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>706</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>2,144</t>
+          <t>843</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>14,413</t>
+          <t>6,321</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
@@ -4140,12 +4140,12 @@
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>904</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>13,440</t>
+          <t>2,543</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="M42" s="10" t="inlineStr">
         <is>
-          <t>947</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N42" s="10" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="P42" s="10" t="inlineStr">
         <is>
-          <t>32,174</t>
+          <t>10,434</t>
         </is>
       </c>
       <c r="Q42" s="10" t="inlineStr">
@@ -4195,24 +4195,24 @@
       </c>
       <c r="R42" s="10" t="inlineStr">
         <is>
-          <t>-676</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="S42" s="10" t="inlineStr">
         <is>
-          <t>-10,273</t>
+          <t>786</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>이지스자산운용</t>
+          <t>칸서스자산운용</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>203</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -4222,12 +4222,12 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>297</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>291</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
@@ -4247,12 +4247,12 @@
       </c>
       <c r="I43" s="10" t="inlineStr">
         <is>
-          <t>4,181</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
         <is>
-          <t>1,287</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K43" s="10" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="P43" s="10" t="inlineStr">
         <is>
-          <t>5,468</t>
+          <t>791</t>
         </is>
       </c>
       <c r="Q43" s="10" t="inlineStr">
@@ -4292,39 +4292,39 @@
       </c>
       <c r="R43" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1</t>
         </is>
       </c>
       <c r="S43" s="10" t="inlineStr">
         <is>
-          <t>-32</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>카디안자산운용</t>
+          <t>케이비자산운용</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>1,405</t>
+          <t>147,146</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>409</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>1,096</t>
+          <t>56,019</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>6,321</t>
+          <t>97,379</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
@@ -4334,17 +4334,17 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>491</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>2,543</t>
+          <t>146,867</t>
         </is>
       </c>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>48,533</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="L44" s="10" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>12,255</t>
         </is>
       </c>
       <c r="M44" s="10" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="P44" s="10" t="inlineStr">
         <is>
-          <t>11,927</t>
+          <t>509,097</t>
         </is>
       </c>
       <c r="Q44" s="10" t="inlineStr">
@@ -4389,39 +4389,39 @@
       </c>
       <c r="R44" s="10" t="inlineStr">
         <is>
-          <t>-16</t>
+          <t>7,527</t>
         </is>
       </c>
       <c r="S44" s="10" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>202,875</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>칸서스자산운용</t>
+          <t>케이씨지아이자산운용</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>7,153</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>195</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>4,010</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>1,787</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>76</t>
         </is>
       </c>
       <c r="H45" s="10" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="P45" s="10" t="inlineStr">
         <is>
-          <t>805</t>
+          <t>13,220</t>
         </is>
       </c>
       <c r="Q45" s="10" t="inlineStr">
@@ -4486,39 +4486,39 @@
       </c>
       <c r="R45" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-22</t>
         </is>
       </c>
       <c r="S45" s="10" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>-1,913</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>케이비자산운용</t>
+          <t>코레이트자산운용</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>203,267</t>
+          <t>133</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>883</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>56,377</t>
+          <t>3,798</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>99,060</t>
+          <t>17,659</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
@@ -4528,22 +4528,22 @@
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>38,618</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>147,121</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>75,161</t>
+          <t>116</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
         <is>
-          <t>529</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K46" s="10" t="inlineStr">
@@ -4553,12 +4553,12 @@
       </c>
       <c r="L46" s="10" t="inlineStr">
         <is>
-          <t>12,255</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M46" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,585</t>
         </is>
       </c>
       <c r="N46" s="10" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="P46" s="10" t="inlineStr">
         <is>
-          <t>633,272</t>
+          <t>30,292</t>
         </is>
       </c>
       <c r="Q46" s="10" t="inlineStr">
@@ -4583,39 +4583,39 @@
       </c>
       <c r="R46" s="10" t="inlineStr">
         <is>
-          <t>6,542</t>
+          <t>-342</t>
         </is>
       </c>
       <c r="S46" s="10" t="inlineStr">
         <is>
-          <t>212,305</t>
+          <t>4,509</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>케이씨지아이자산운용</t>
+          <t>키움투자자산운용</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>9,955</t>
+          <t>35,965</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>725</t>
+          <t>59</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>4,010</t>
+          <t>2,687</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>1,787</t>
+          <t>35,018</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
@@ -4625,22 +4625,22 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>8,965</t>
+          <t>4,553</t>
         </is>
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71,084</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K47" s="10" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="P47" s="10" t="inlineStr">
         <is>
-          <t>25,525</t>
+          <t>153,366</t>
         </is>
       </c>
       <c r="Q47" s="10" t="inlineStr">
@@ -4680,24 +4680,24 @@
       </c>
       <c r="R47" s="10" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>3,707</t>
         </is>
       </c>
       <c r="S47" s="10" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>9,780</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>코레이트자산운용</t>
+          <t>타임폴리오자산운용</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>23,943</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>3,798</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E48" s="10" t="inlineStr">
         <is>
-          <t>17,659</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9,234</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J48" s="10" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="M48" s="10" t="inlineStr">
         <is>
-          <t>8,585</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N48" s="10" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="P48" s="10" t="inlineStr">
         <is>
-          <t>30,313</t>
+          <t>33,177</t>
         </is>
       </c>
       <c r="Q48" s="10" t="inlineStr">
@@ -4777,39 +4777,39 @@
       </c>
       <c r="R48" s="10" t="inlineStr">
         <is>
-          <t>-342</t>
+          <t>382</t>
         </is>
       </c>
       <c r="S48" s="10" t="inlineStr">
         <is>
-          <t>4,506</t>
+          <t>18,759</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>키움투자자산운용</t>
+          <t>트러스톤자산운용</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>45,708</t>
+          <t>2,103</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>196</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>2,897</t>
+          <t>918</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>35,018</t>
+          <t>3,357</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
@@ -4819,17 +4819,17 @@
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>17,836</t>
+          <t>38</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
         <is>
-          <t>71,084</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
         <is>
-          <t>7,490</t>
+          <t>370</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="P49" s="10" t="inlineStr">
         <is>
-          <t>180,093</t>
+          <t>6,984</t>
         </is>
       </c>
       <c r="Q49" s="10" t="inlineStr">
@@ -4874,39 +4874,39 @@
       </c>
       <c r="R49" s="10" t="inlineStr">
         <is>
-          <t>3,428</t>
+          <t>5</t>
         </is>
       </c>
       <c r="S49" s="10" t="inlineStr">
         <is>
-          <t>8,237</t>
+          <t>-95</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>타임폴리오자산운용</t>
+          <t>플러스자산운용</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>81,919</t>
+          <t>167</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>64</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>4,304</t>
+          <t>152</t>
         </is>
       </c>
       <c r="E50" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>296</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
@@ -4916,12 +4916,12 @@
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>10,160</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>52,942</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="P50" s="10" t="inlineStr">
         <is>
-          <t>96,383</t>
+          <t>53,619</t>
         </is>
       </c>
       <c r="Q50" s="10" t="inlineStr">
@@ -4971,39 +4971,39 @@
       </c>
       <c r="R50" s="10" t="inlineStr">
         <is>
-          <t>-684</t>
+          <t>133</t>
         </is>
       </c>
       <c r="S50" s="10" t="inlineStr">
         <is>
-          <t>53,227</t>
+          <t>22,912</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>트러스톤자산운용</t>
+          <t>피델리티자산운용</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>2,324</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>3,421</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>90</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="I51" s="10" t="inlineStr">
         <is>
-          <t>370</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J51" s="10" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="P51" s="10" t="inlineStr">
         <is>
-          <t>7,517</t>
+          <t>90</t>
         </is>
       </c>
       <c r="Q51" s="10" t="inlineStr">
@@ -5068,39 +5068,39 @@
       </c>
       <c r="R51" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S51" s="10" t="inlineStr">
         <is>
-          <t>-66</t>
+          <t>-8</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>플러스자산운용</t>
+          <t>하나대체투자자산운용</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>52,942</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
@@ -5125,7 +5125,7 @@
       </c>
       <c r="J52" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>738</t>
         </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="P52" s="10" t="inlineStr">
         <is>
-          <t>53,619</t>
+          <t>738</t>
         </is>
       </c>
       <c r="Q52" s="10" t="inlineStr">
@@ -5165,39 +5165,39 @@
       </c>
       <c r="R52" s="10" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S52" s="10" t="inlineStr">
         <is>
-          <t>22,912</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>피델리티자산운용</t>
+          <t>하나자산운용</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>1,050</t>
+          <t>16,119</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,824</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,325</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>30,113</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
@@ -5207,17 +5207,17 @@
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>28,497</t>
+          <t>1,524</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>119,267</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,743</t>
         </is>
       </c>
       <c r="J53" s="10" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="L53" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3,720</t>
         </is>
       </c>
       <c r="M53" s="10" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="P53" s="10" t="inlineStr">
         <is>
-          <t>29,547</t>
+          <t>179,635</t>
         </is>
       </c>
       <c r="Q53" s="10" t="inlineStr">
@@ -5262,19 +5262,19 @@
       </c>
       <c r="R53" s="10" t="inlineStr">
         <is>
-          <t>-40</t>
+          <t>1,420</t>
         </is>
       </c>
       <c r="S53" s="10" t="inlineStr">
         <is>
-          <t>-6,177</t>
+          <t>37,047</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>하나대체투자자산운용</t>
+          <t>한국투자리얼에셋운용</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
@@ -5314,12 +5314,12 @@
       </c>
       <c r="I54" s="10" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J54" s="10" t="inlineStr">
         <is>
-          <t>2,104</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K54" s="10" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="P54" s="10" t="inlineStr">
         <is>
-          <t>2,514</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q54" s="10" t="inlineStr">
@@ -5364,34 +5364,34 @@
       </c>
       <c r="S54" s="10" t="inlineStr">
         <is>
-          <t>-515</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>하나자산운용</t>
+          <t>한국투자밸류자산운용</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>28,522</t>
+          <t>8,573</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>2,824</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>9,061</t>
+          <t>7,689</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>30,113</t>
+          <t>412</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
@@ -5401,22 +5401,22 @@
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>6,372</t>
+          <t>4,639</t>
         </is>
       </c>
       <c r="H55" s="10" t="inlineStr">
         <is>
-          <t>119,325</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I55" s="10" t="inlineStr">
         <is>
-          <t>2,743</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J55" s="10" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K55" s="10" t="inlineStr">
@@ -5426,12 +5426,12 @@
       </c>
       <c r="L55" s="10" t="inlineStr">
         <is>
-          <t>4,292</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M55" s="10" t="inlineStr">
         <is>
-          <t>1,004</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N55" s="10" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="P55" s="10" t="inlineStr">
         <is>
-          <t>204,703</t>
+          <t>21,314</t>
         </is>
       </c>
       <c r="Q55" s="10" t="inlineStr">
@@ -5456,39 +5456,39 @@
       </c>
       <c r="R55" s="10" t="inlineStr">
         <is>
-          <t>1,237</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="S55" s="10" t="inlineStr">
         <is>
-          <t>46,537</t>
+          <t>1,215</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>한국투자리얼에셋운용</t>
+          <t>한국투자신탁운용</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>64,393</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,996</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,776</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53,683</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
@@ -5498,22 +5498,22 @@
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,112</t>
         </is>
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>59,724</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>2,388</t>
+          <t>7,842</t>
         </is>
       </c>
       <c r="J56" s="10" t="inlineStr">
         <is>
-          <t>1,933</t>
+          <t>170</t>
         </is>
       </c>
       <c r="K56" s="10" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="L56" s="10" t="inlineStr">
         <is>
-          <t>1,769</t>
+          <t>42,352</t>
         </is>
       </c>
       <c r="M56" s="10" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="P56" s="10" t="inlineStr">
         <is>
-          <t>6,090</t>
+          <t>240,048</t>
         </is>
       </c>
       <c r="Q56" s="10" t="inlineStr">
@@ -5553,39 +5553,39 @@
       </c>
       <c r="R56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,941</t>
         </is>
       </c>
       <c r="S56" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>51,329</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>한국투자밸류자산운용</t>
+          <t>한화자산운용</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>8,834</t>
+          <t>73,794</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>134</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>7,689</t>
+          <t>843</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>27,205</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
@@ -5595,22 +5595,22 @@
       </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
-          <t>4,639</t>
+          <t>322</t>
         </is>
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>50,964</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,815</t>
         </is>
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>76</t>
         </is>
       </c>
       <c r="K57" s="10" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="L57" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>168</t>
         </is>
       </c>
       <c r="M57" s="10" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="P57" s="10" t="inlineStr">
         <is>
-          <t>21,574</t>
+          <t>167,321</t>
         </is>
       </c>
       <c r="Q57" s="10" t="inlineStr">
@@ -5650,39 +5650,39 @@
       </c>
       <c r="R57" s="10" t="inlineStr">
         <is>
-          <t>-15</t>
+          <t>2,036</t>
         </is>
       </c>
       <c r="S57" s="10" t="inlineStr">
         <is>
-          <t>1,247</t>
+          <t>40,360</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>한국투자신탁운용</t>
+          <t>현대인베스트먼트자산운용</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>228,186</t>
+          <t>345</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>5,545</t>
+          <t>799</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>27,723</t>
+          <t>433</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
         <is>
-          <t>76,179</t>
+          <t>1,317</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
@@ -5692,22 +5692,22 @@
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>52,269</t>
+          <t>18</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>65,115</t>
+          <t>21,717</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
         <is>
-          <t>24,996</t>
+          <t>142</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K58" s="10" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="L58" s="10" t="inlineStr">
         <is>
-          <t>42,378</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M58" s="10" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="P58" s="10" t="inlineStr">
         <is>
-          <t>522,633</t>
+          <t>24,771</t>
         </is>
       </c>
       <c r="Q58" s="10" t="inlineStr">
@@ -5747,39 +5747,39 @@
       </c>
       <c r="R58" s="10" t="inlineStr">
         <is>
-          <t>-657</t>
+          <t>265</t>
         </is>
       </c>
       <c r="S58" s="10" t="inlineStr">
         <is>
-          <t>81,741</t>
+          <t>4,726</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>한화자산운용</t>
+          <t>현대자산운용</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>97,479</t>
+          <t>2,513</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>1,570</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>28,416</t>
+          <t>213</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
@@ -5789,22 +5789,22 @@
       </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
-          <t>11,985</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>50,964</t>
+          <t>15,955</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr">
         <is>
-          <t>18,335</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J59" s="10" t="inlineStr">
         <is>
-          <t>286</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K59" s="10" t="inlineStr">
@@ -5814,12 +5814,12 @@
       </c>
       <c r="L59" s="10" t="inlineStr">
         <is>
-          <t>446</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M59" s="10" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N59" s="10" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="P59" s="10" t="inlineStr">
         <is>
-          <t>209,660</t>
+          <t>18,721</t>
         </is>
       </c>
       <c r="Q59" s="10" t="inlineStr">
@@ -5844,39 +5844,39 @@
       </c>
       <c r="R59" s="10" t="inlineStr">
         <is>
-          <t>1,937</t>
+          <t>-298</t>
         </is>
       </c>
       <c r="S59" s="10" t="inlineStr">
         <is>
-          <t>60,180</t>
+          <t>464</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>현대인베스트먼트자산운용</t>
+          <t>흥국자산운용</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>1,827</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>799</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>2,205</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>1,317</t>
+          <t>20,121</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
@@ -5886,17 +5886,17 @@
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>21,717</t>
+          <t>14,156</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>5,580</t>
         </is>
       </c>
       <c r="J60" s="10" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="M60" s="10" t="inlineStr">
         <is>
-          <t>638</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N60" s="10" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="P60" s="10" t="inlineStr">
         <is>
-          <t>25,951</t>
+          <t>43,889</t>
         </is>
       </c>
       <c r="Q60" s="10" t="inlineStr">
@@ -5941,39 +5941,39 @@
       </c>
       <c r="R60" s="10" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>86</t>
         </is>
       </c>
       <c r="S60" s="10" t="inlineStr">
         <is>
-          <t>5,368</t>
+          <t>-6,224</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>현대자산운용</t>
+          <t>자산운용- 소계</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>2,513</t>
+          <t>2,034,815</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>22,491</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>188,994</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>807,824</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
@@ -5983,22 +5983,22 @@
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>35,355</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>15,955</t>
+          <t>1,642,609</t>
         </is>
       </c>
       <c r="I61" s="10" t="inlineStr">
         <is>
-          <t>523</t>
+          <t>761,630</t>
         </is>
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9,118</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
@@ -6008,17 +6008,17 @@
       </c>
       <c r="L61" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>105,133</t>
         </is>
       </c>
       <c r="M61" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26,085</t>
         </is>
       </c>
       <c r="N61" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>360</t>
         </is>
       </c>
       <c r="O61" s="10" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="P61" s="10" t="inlineStr">
         <is>
-          <t>19,272</t>
+          <t>5,634,414</t>
         </is>
       </c>
       <c r="Q61" s="10" t="inlineStr">
@@ -6038,39 +6038,39 @@
       </c>
       <c r="R61" s="10" t="inlineStr">
         <is>
-          <t>-298</t>
+          <t>50,706</t>
         </is>
       </c>
       <c r="S61" s="10" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>1,787,252</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>흥국자산운용</t>
+          <t>합계</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>1,831</t>
+          <t>2,034,815</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,491</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>2,205</t>
+          <t>188,994</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>20,121</t>
+          <t>807,824</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
@@ -6080,22 +6080,22 @@
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>603</t>
+          <t>35,355</t>
         </is>
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>14,156</t>
+          <t>1,642,609</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr">
         <is>
-          <t>5,580</t>
+          <t>761,630</t>
         </is>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>9,118</t>
         </is>
       </c>
       <c r="K62" s="10" t="inlineStr">
@@ -6105,17 +6105,17 @@
       </c>
       <c r="L62" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>105,133</t>
         </is>
       </c>
       <c r="M62" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26,085</t>
         </is>
       </c>
       <c r="N62" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>360</t>
         </is>
       </c>
       <c r="O62" s="10" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="P62" s="10" t="inlineStr">
         <is>
-          <t>44,523</t>
+          <t>5,634,414</t>
         </is>
       </c>
       <c r="Q62" s="10" t="inlineStr">
@@ -6135,206 +6135,12 @@
       </c>
       <c r="R62" s="10" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>50,706</t>
         </is>
       </c>
       <c r="S62" s="10" t="inlineStr">
         <is>
-          <t>-6,377</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>자산운용- 소계</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>3,312,791</t>
-        </is>
-      </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>40,897</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>261,539</t>
-        </is>
-      </c>
-      <c r="E63" s="10" t="inlineStr">
-        <is>
-          <t>869,241</t>
-        </is>
-      </c>
-      <c r="F63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G63" s="10" t="inlineStr">
-        <is>
-          <t>359,655</t>
-        </is>
-      </c>
-      <c r="H63" s="10" t="inlineStr">
-        <is>
-          <t>1,664,309</t>
-        </is>
-      </c>
-      <c r="I63" s="10" t="inlineStr">
-        <is>
-          <t>1,066,606</t>
-        </is>
-      </c>
-      <c r="J63" s="10" t="inlineStr">
-        <is>
-          <t>21,073</t>
-        </is>
-      </c>
-      <c r="K63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L63" s="10" t="inlineStr">
-        <is>
-          <t>112,159</t>
-        </is>
-      </c>
-      <c r="M63" s="10" t="inlineStr">
-        <is>
-          <t>93,079</t>
-        </is>
-      </c>
-      <c r="N63" s="10" t="inlineStr">
-        <is>
-          <t>360</t>
-        </is>
-      </c>
-      <c r="O63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P63" s="10" t="inlineStr">
-        <is>
-          <t>7,801,709</t>
-        </is>
-      </c>
-      <c r="Q63" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R63" s="10" t="inlineStr">
-        <is>
-          <t>29,176</t>
-        </is>
-      </c>
-      <c r="S63" s="10" t="inlineStr">
-        <is>
-          <t>2,207,774</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>합계</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>3,312,791</t>
-        </is>
-      </c>
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>40,897</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>261,539</t>
-        </is>
-      </c>
-      <c r="E64" s="10" t="inlineStr">
-        <is>
-          <t>869,241</t>
-        </is>
-      </c>
-      <c r="F64" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="10" t="inlineStr">
-        <is>
-          <t>359,655</t>
-        </is>
-      </c>
-      <c r="H64" s="10" t="inlineStr">
-        <is>
-          <t>1,664,309</t>
-        </is>
-      </c>
-      <c r="I64" s="10" t="inlineStr">
-        <is>
-          <t>1,066,606</t>
-        </is>
-      </c>
-      <c r="J64" s="10" t="inlineStr">
-        <is>
-          <t>21,073</t>
-        </is>
-      </c>
-      <c r="K64" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L64" s="10" t="inlineStr">
-        <is>
-          <t>112,159</t>
-        </is>
-      </c>
-      <c r="M64" s="10" t="inlineStr">
-        <is>
-          <t>93,079</t>
-        </is>
-      </c>
-      <c r="N64" s="10" t="inlineStr">
-        <is>
-          <t>360</t>
-        </is>
-      </c>
-      <c r="O64" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P64" s="10" t="inlineStr">
-        <is>
-          <t>7,801,709</t>
-        </is>
-      </c>
-      <c r="Q64" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R64" s="10" t="inlineStr">
-        <is>
-          <t>29,176</t>
-        </is>
-      </c>
-      <c r="S64" s="10" t="inlineStr">
-        <is>
-          <t>2,207,774</t>
+          <t>1,787,252</t>
         </is>
       </c>
     </row>

</xml_diff>